<commit_message>
feat: add 2 new tech articles + covers + update content plan
</commit_message>
<xml_diff>
--- a/content-plan-lofa.xlsx
+++ b/content-plan-lofa.xlsx
@@ -1182,10 +1182,14 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>BATCH 2</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr"/>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Tombol keyboard mekanik tiba-tiba mengetik dua huruf? Simak penyebab umum double input dan cara mengatasinya langkah demi langkah.</t>
@@ -1244,10 +1248,14 @@
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>BATCH 2</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr"/>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
           <t>Keyboard tidak terdeteksi di Windows bisa bikin panik. Simak langkah diagnosis dan solusi untuk membuat keyboard kembali berfungsi.</t>

</xml_diff>

<commit_message>
GSC: meta tag verifikasi
</commit_message>
<xml_diff>
--- a/content-plan-lofa.xlsx
+++ b/content-plan-lofa.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2706,6 +2706,486 @@
       <c r="N36" s="4" t="inlineStr">
         <is>
           <t>Batch 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Game/PC</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Perkembangan Game Terbaru 2025: Apa yang Baru di Industri Gaming?</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>perkembangan-game-terbaru-2025</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>tech</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>BATCH 7</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Industri gaming berkembang cepat. Simak perkembangan game terbaru 2025: rilis AAA, trend indie, teknologi cloud gaming, dan AI di game.</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>game, gaming, 2025, industri, rilis</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>tips-trik-game-pc-pemula</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>new video game releases 2025 gaming setup</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Batch 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Game/PC</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Tips Trik Game PC untuk Pemula: Naikkan Skill &amp; Performa</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>tips-trik-game-pc-pemula</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>tech</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Informational/Problem solving</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>BATCH 7</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Baru main game di PC? Simak tips trik game PC untuk pemula: setting grafis optimal, shortcut berguna, dan cara naikkan FPS tanpa upgrade hardware.</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>game, pc, tips, trik, pemula, fps</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>komponen-pc-gaming-murah-meriah</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>pc gaming tips tricks settings optimization</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Batch 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Game/PC</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Panduan Komponen PC Gaming Murah Meriah 2025</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>komponen-pc-gaming-murah-meriah</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>tech</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Informational/Commercial</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>BATCH 7</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Mau rakit PC gaming tapi budget terbatas? Simak panduan komponen PC gaming murah meriah 2025: CPU, GPU, RAM, SSD, PSU, casing yang value for money.</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>pc, gaming, rakit, budget, komponen</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>tips-trik-game-pc-pemula</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>budget gaming pc components build 2025</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Batch 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Game/PC</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Cara Memilih GPU untuk Gaming: NVIDIA vs AMD 2025</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>cara-memilih-gpu-gaming-nvidia-vs-amd</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>tech</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>BATCH 7</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>NVIDIA RTX vs AMD Radeon: mana GPU gaming terbaik 2025? Bandingkan performa, fitur (DLSS vs FSR), ray tracing, dan harga per tier.</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>gpu, nvidia, amd, gaming, perbandingan</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>komponen-pc-gaming-murah-meriah</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>nvidia rtx amd radeon gpu comparison 2025</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Batch 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Game/PC</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>SSD vs HDD untuk Gaming: Mana yang Lebih Cepat Load Game?</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>ssd-vs-hdd-gaming</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>tech</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>BATCH 7</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>SSD NVMe, SSD SATA, atau HDD untuk gaming? Simak perbandingan kecepatan load game, kapasitas per rupiah, dan rekomendasi storage terbaik 2025.</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>ssd, hdd, storage, gaming, load time</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>cara-mengecek-kesehatan-ssd-di-windows</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>ssd vs hdd gaming loading speed comparison</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Batch 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Game/PC</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Cara Mengoptimalkan Windows 11 untuk Gaming</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>cara-mengoptimalkan-windows-11-gaming</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>tech</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Problem solving</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>BATCH 7</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Windows 11 bisa lebih cepat untuk gaming. Simak cara mengoptimalkan: Game Mode, GPU scheduling, power plan, disable service tidak perlu, dan tweak registry.</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>windows 11, gaming, optimasi, game mode</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>cara-membuat-windows-11-lebih-ringan</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>windows 11 gaming optimization settings</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Batch 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Game/PC</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Monitor Gaming: Refresh Rate, Response Time, Panel Mana yang Dipilih?</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>monitor-gaming-refresh-rate-response-time-panel</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>tech</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Informational/Commercial</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>BATCH 7</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Bingung pilih monitor gaming? Pahami refresh rate (144Hz/240Hz/360Hz), response time (1ms/0.5ms), panel IPS/VA/TN/OLED, dan resolusi 1080p/1440p/4K.</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>monitor, gaming, refresh rate, panel, ips</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>komponen-pc-gaming-murah-meriah</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>gaming monitor refresh rate ips va oled comparison</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Batch 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Game/PC</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Perbedaan Mechanical vs Membrane Keyboard untuk Gaming</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>perbedaan-mechanical-membrane-keyboard-gaming</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>tech</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>BATCH 7</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Keyboard mechanical vs membrane untuk gaming: mana lebih cepat respons, awet, dan nyaman? Simak perbandingan switch, actuation point, dan rekomendasi budget.</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>keyboard, mechanical, membrane, gaming</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>mechanical-keyboard-vs-membrane</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>mechanical vs membrane keyboard gaming comparison</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Batch 7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build: add new article Cara Mengatasi WiFi Laptop Tidak Terhubung (auto post tech)
</commit_message>
<xml_diff>
--- a/content-plan-lofa.xlsx
+++ b/content-plan-lofa.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:P44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -590,6 +590,16 @@
           <t>Catatan</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Keyword Produk Affiliate</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Posted to Blog</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -660,6 +670,16 @@
           <t>Artikel lama, tetap live</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard hot swap</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -730,6 +750,16 @@
           <t>Artikel lama, tetap live</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard hot swap</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -800,6 +830,16 @@
           <t>Artikel lama, tetap live</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>wadah sayuran / kotak penyimpanan</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -832,7 +872,7 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>BATCH 1</t>
+          <t>LIVE</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -868,6 +908,16 @@
       <c r="N7" s="4" t="inlineStr">
         <is>
           <t>Batch 1</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard hot swap</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -902,7 +952,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>BATCH 1</t>
+          <t>LIVE</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -938,6 +988,16 @@
       <c r="N8" s="4" t="inlineStr">
         <is>
           <t>Batch 1</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard hot swap</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -972,7 +1032,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>BATCH 1</t>
+          <t>LIVE</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1008,6 +1068,16 @@
       <c r="N9" s="4" t="inlineStr">
         <is>
           <t>Batch 1</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard hot swap</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1112,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>BATCH 1</t>
+          <t>LIVE</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1078,6 +1148,16 @@
       <c r="N10" s="4" t="inlineStr">
         <is>
           <t>Batch 1</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard hot swap</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1192,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>BATCH 1</t>
+          <t>LIVE</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1148,6 +1228,16 @@
       <c r="N11" s="4" t="inlineStr">
         <is>
           <t>Batch 1</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard hot swap</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1216,6 +1306,16 @@
           <t>Batch 2 — menunggu approval</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard hot swap</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1282,6 +1382,16 @@
           <t>Batch 2</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard hot swap</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1314,10 +1424,14 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>BATCH 2</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr"/>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Satu atau beberapa tombol keyboard mechanical tidak merespons? Simak penyebab umum dan langkah perbaikan yang bisa dicoba sendiri.</t>
@@ -1338,10 +1452,24 @@
           <t>keyboard single key not working closeup</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>cover-cara-mengatasi-tombol-keyboard-mechanical-tidak-berfungsi.jpg</t>
+        </is>
+      </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
           <t>Batch 2</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard hot swap</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1376,10 +1504,14 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>BATCH 2</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr"/>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Seberapa sering keyboard mechanical perlu dibersihkan? Simak panduan jadwal perawatan berdasarkan intensitas pemakaian dan lingkungan.</t>
@@ -1400,10 +1532,24 @@
           <t>clean keyboard routine maintenance workspace</t>
         </is>
       </c>
-      <c r="M15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>cover-seberapa-sering-keyboard-mechanical-dibersihkan.jpg</t>
+        </is>
+      </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
           <t>Batch 2</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard hot swap</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1438,10 +1584,14 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>BATCH 2</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr"/>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Membersihkan keyboard dengan alkohol bisa merusak switch dan keycap jika salah. Simak apa yang aman dan apa yang sebaiknya dihindari.</t>
@@ -1462,10 +1612,24 @@
           <t>isopropyl alcohol cleaning electronics keyboard</t>
         </is>
       </c>
-      <c r="M16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>cover-bolehkah-membersihkan-keyboard-mechanical-dengan-alkohol.jpg</t>
+        </is>
+      </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
           <t>Batch 2</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard hot swap</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1500,10 +1664,14 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>BATCH 3</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr"/>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
           <t>Laptop terasa lambat saat menyala? Matikan aplikasi startup yang tidak perlu di Windows 11 dengan langkah sederhana ini.</t>
@@ -1524,10 +1692,24 @@
           <t>windows task manager startup apps</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>cover-cara-mematikan-startup-apps-windows-11.jpg</t>
+        </is>
+      </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
           <t>Batch 3</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>ssd laptop / ram laptop</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1562,10 +1744,14 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>BATCH 3</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr"/>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Storage penuh? Simak cara membersihkan file sampah, cache, dan file besar di Windows 11 tanpa aplikasi tambahan.</t>
@@ -1586,10 +1772,24 @@
           <t>windows disk cleanup storage settings</t>
         </is>
       </c>
-      <c r="M18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>cover-cara-membersihkan-storage-windows-11.jpg</t>
+        </is>
+      </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
           <t>Batch 3</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>ssd laptop / ram laptop</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1624,10 +1824,14 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>BATCH 3</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr"/>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
           <t>Cek kesehatan SSD penting agar data aman. Simak cara memeriksa kondisi SSD di Windows dengan tools bawaan dan pihak ketiga.</t>
@@ -1648,10 +1852,24 @@
           <t>ssd drive health check laptop</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr"/>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>cover-cara-mengecek-kesehatan-ssd-di-windows.jpg</t>
+        </is>
+      </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
           <t>Batch 3</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>ssd laptop / ram laptop</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1686,10 +1904,14 @@
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>BATCH 3</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr"/>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Ingin tahu kapasitas dan pemakaian RAM laptop? Simak cara mengecek spesifikasi RAM di Windows dengan beberapa metode mudah.</t>
@@ -1710,10 +1932,24 @@
           <t>laptop ram memory module closeup</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>cover-cara-mengecek-ram-laptop-di-windows.jpg</t>
+        </is>
+      </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
           <t>Batch 3</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>ssd laptop / ram laptop</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1778,6 +2014,16 @@
           <t>Batch 3</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>ssd laptop / ram laptop</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1840,6 +2086,16 @@
           <t>Batch 3</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>ssd laptop / ram laptop</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1902,6 +2158,16 @@
           <t>Batch 3</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>ssd laptop / ram laptop</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1964,6 +2230,16 @@
           <t>Batch 3</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>ssd laptop / ram laptop</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -2026,6 +2302,16 @@
           <t>Batch 4</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>cooling pad laptop / thermal paste</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -2088,6 +2374,16 @@
           <t>Batch 4</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>cooling pad laptop / thermal paste</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -2150,6 +2446,16 @@
           <t>Batch 4</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>cooling pad laptop / thermal paste</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -2212,6 +2518,16 @@
           <t>Batch 4</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>cooling pad laptop / thermal paste</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -2274,6 +2590,16 @@
           <t>Batch 5</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>wadah sayuran / kotak penyimpanan</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -2336,6 +2662,16 @@
           <t>Batch 5</t>
         </is>
       </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>wadah sayuran / kotak penyimpanan</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -2398,6 +2734,16 @@
           <t>Batch 5</t>
         </is>
       </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>wadah sayuran / kotak penyimpanan</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -2460,6 +2806,16 @@
           <t>Batch 5</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>wadah sayuran / kotak penyimpanan</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -2522,6 +2878,16 @@
           <t>Batch 6</t>
         </is>
       </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>wadah sayuran / kotak penyimpanan</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -2584,6 +2950,16 @@
           <t>Batch 6</t>
         </is>
       </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>wadah sayuran / kotak penyimpanan</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -2646,6 +3022,16 @@
           <t>Batch 6</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>wadah sayuran / kotak penyimpanan</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -2708,6 +3094,16 @@
           <t>Batch 6</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>wadah sayuran / kotak penyimpanan</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2763,9 +3159,24 @@
           <t>new video game releases 2025 gaming setup</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>cover-perkembangan-game-2025.jpg</t>
+        </is>
+      </c>
       <c r="N37" t="inlineStr">
         <is>
           <t>Batch 7</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>game / gaming pc</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2823,9 +3234,24 @@
           <t>pc gaming tips tricks settings optimization</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>cover-tips-trik-game-pc-pemula.jpg</t>
+        </is>
+      </c>
       <c r="N38" t="inlineStr">
         <is>
           <t>Batch 7</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>game pc / gaming mouse</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2883,9 +3309,24 @@
           <t>budget gaming pc components build 2025</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>cover-komponen-pc-gaming-murah.jpg</t>
+        </is>
+      </c>
       <c r="N39" t="inlineStr">
         <is>
           <t>Batch 7</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>cpu amd ryzen / gpu nvidia rtx / ram ddr4</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2943,9 +3384,24 @@
           <t>nvidia rtx amd radeon gpu comparison 2025</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>cover-gpu-nvidia-vs-amd-gaming.jpg</t>
+        </is>
+      </c>
       <c r="N40" t="inlineStr">
         <is>
           <t>Batch 7</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>gpu nvidia rtx / gpu amd radeon</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -3003,9 +3459,24 @@
           <t>ssd vs hdd gaming loading speed comparison</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>cover-ssd-vs-hdd-gaming.jpg</t>
+        </is>
+      </c>
       <c r="N41" t="inlineStr">
         <is>
           <t>Batch 7</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>ssd nvme / hdd</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -3063,9 +3534,24 @@
           <t>windows 11 gaming optimization settings</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>cover-windows-11-gaming-optimization.jpg</t>
+        </is>
+      </c>
       <c r="N42" t="inlineStr">
         <is>
           <t>Batch 7</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>windows 11 / ssd laptop</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -3123,9 +3609,24 @@
           <t>gaming monitor refresh rate ips va oled comparison</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>cover-monitor-gaming-refresh-rate.jpg</t>
+        </is>
+      </c>
       <c r="N43" t="inlineStr">
         <is>
           <t>Batch 7</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>monitor gaming ips / monitor gaming va</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -3183,9 +3684,24 @@
           <t>mechanical vs membrane keyboard gaming comparison</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>cover-mechanical-vs-membrane-gaming.jpg</t>
+        </is>
+      </c>
       <c r="N44" t="inlineStr">
         <is>
           <t>Batch 7</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>keyboard mechanical / keyboard gaming</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>